<commit_message>
Fixed incorrect PN on 5.1K resistors.
</commit_message>
<xml_diff>
--- a/HARDWARE/KICAD/Fabrication/ColorTemp Rev.00 - BOM (JLCPCB).xlsx
+++ b/HARDWARE/KICAD/Fabrication/ColorTemp Rev.00 - BOM (JLCPCB).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Andre\ENGINEERING\PROJECTS\MECHATRONIX LAB\ColorTemp\HARDWARE\KICAD\Fabrication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447EECC6-D186-4B29-B159-EE5EBC6CF542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD57EA5-E88C-4712-BEB2-DEDCFE7513E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15345" yWindow="-13605" windowWidth="21600" windowHeight="11295" xr2:uid="{7EA92FB2-F55C-44C2-BB28-0C1A7EE98431}"/>
+    <workbookView xWindow="-8640" yWindow="-16410" windowWidth="21600" windowHeight="11295" xr2:uid="{7EA92FB2-F55C-44C2-BB28-0C1A7EE98431}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -137,9 +137,6 @@
     <t>C2927029</t>
   </si>
   <si>
-    <t>C11702</t>
-  </si>
-  <si>
     <t>C25091</t>
   </si>
   <si>
@@ -156,6 +153,9 @@
   </si>
   <si>
     <t>C4154880</t>
+  </si>
+  <si>
+    <t>C25905</t>
   </si>
 </sst>
 </file>
@@ -580,16 +580,16 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
       </c>
       <c r="C4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
         <v>38</v>
-      </c>
-      <c r="D4" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -617,7 +617,7 @@
         <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -631,7 +631,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -645,7 +645,7 @@
         <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -659,7 +659,7 @@
         <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -673,7 +673,7 @@
         <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -687,7 +687,7 @@
         <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>